<commit_message>
Add Flights tab with flight schedule from location.xlsx
</commit_message>
<xml_diff>
--- a/location.xlsx
+++ b/location.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\technology\repositories\antigravity\guangzhou\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D773D417-5E57-4757-B8A4-7A72535C4E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D31EBF-6B96-40C0-B8C0-662DFA2D0C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="itinerary" sheetId="2" r:id="rId1"/>
-    <sheet name="location" sheetId="1" r:id="rId2"/>
+    <sheet name="flight" sheetId="3" r:id="rId1"/>
+    <sheet name="itinerary" sheetId="2" r:id="rId2"/>
+    <sheet name="location" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="133">
   <si>
     <t>Location</t>
   </si>
@@ -416,6 +417,48 @@
   </si>
   <si>
     <t xml:space="preserve">DAY 5 – SUN, JAN 17 (SHOPPING + DEPARTURE) </t>
+  </si>
+  <si>
+    <t>flight no</t>
+  </si>
+  <si>
+    <t>date from</t>
+  </si>
+  <si>
+    <t>date to</t>
+  </si>
+  <si>
+    <t>from</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to </t>
+  </si>
+  <si>
+    <t>CZ354</t>
+  </si>
+  <si>
+    <t>cz351</t>
+  </si>
+  <si>
+    <t>13/1/2027 - 13:40</t>
+  </si>
+  <si>
+    <t>13/1/2027 - 17:40</t>
+  </si>
+  <si>
+    <t>17/1/2027 - 18:50</t>
+  </si>
+  <si>
+    <t>17/1/2027 - 23:00</t>
+  </si>
+  <si>
+    <t>Singapore</t>
+  </si>
+  <si>
+    <t>Guangzhou</t>
+  </si>
+  <si>
+    <t>GuangZhou</t>
   </si>
 </sst>
 </file>
@@ -510,7 +553,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -537,6 +580,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -817,6 +861,67 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AED1DDF-C5A8-4CC0-AA88-5D84973396B3}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD85DFBA-C2AF-4F01-8853-00C589EED3EF}">
   <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1291,7 +1396,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Add inter-location transit directions (Metro, DiDi, Walk) and update hotel to CityNote Hotel
</commit_message>
<xml_diff>
--- a/location.xlsx
+++ b/location.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\technology\repositories\antigravity\guangzhou\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D31EBF-6B96-40C0-B8C0-662DFA2D0C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D08BCA5-7CE5-45FA-BD6D-833CBE68386E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="flight" sheetId="3" r:id="rId1"/>
@@ -248,9 +248,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Check in at Kspace</t>
-  </si>
-  <si>
     <t>Freshen up</t>
   </si>
   <si>
@@ -299,9 +296,6 @@
     <t>80–150 RMB</t>
   </si>
   <si>
-    <t>Back to Kspace</t>
-  </si>
-  <si>
     <t>Walk or taxi</t>
   </si>
   <si>
@@ -350,9 +344,6 @@
     <t>Climb pagoda for views</t>
   </si>
   <si>
-    <t>Back to Kspace – rest</t>
-  </si>
-  <si>
     <t>Chill time</t>
   </si>
   <si>
@@ -383,9 +374,6 @@
     <t>Lunch at mall</t>
   </si>
   <si>
-    <t>Back to Kspace – pick up luggage</t>
-  </si>
-  <si>
     <t>Metro to Airport North</t>
   </si>
   <si>
@@ -459,6 +447,18 @@
   </si>
   <si>
     <t>GuangZhou</t>
+  </si>
+  <si>
+    <t>Check in at CityNote</t>
+  </si>
+  <si>
+    <t>Back to CityNote</t>
+  </si>
+  <si>
+    <t>Back to CityNote – rest</t>
+  </si>
+  <si>
+    <t>Back to CityNote – pick up luggage</t>
   </si>
 </sst>
 </file>
@@ -867,53 +867,53 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E1" t="s">
         <v>119</v>
-      </c>
-      <c r="B1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D2" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="E2" t="s">
         <v>127</v>
-      </c>
-      <c r="D2" t="s">
-        <v>130</v>
-      </c>
-      <c r="E2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="D3" t="s">
         <v>128</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="D3" t="s">
-        <v>132</v>
-      </c>
       <c r="E3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -933,7 +933,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -953,11 +953,11 @@
       <c r="A3" s="8">
         <v>0.8125</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>62</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -965,10 +965,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>64</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -979,7 +979,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -987,10 +987,10 @@
         <v>0.9375</v>
       </c>
       <c r="B6" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>67</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1000,7 +1000,7 @@
     </row>
     <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1024,7 +1024,7 @@
         <v>11</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1032,10 +1032,10 @@
         <v>0.5</v>
       </c>
       <c r="B11" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>70</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1043,10 +1043,10 @@
         <v>0.5625</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -1057,7 +1057,7 @@
         <v>18</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1065,10 +1065,10 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="B14" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>75</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1076,10 +1076,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="B15" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -1087,10 +1087,10 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>79</v>
+        <v>130</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1100,7 +1100,7 @@
     </row>
     <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1124,7 +1124,7 @@
         <v>25</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1132,10 +1132,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1143,10 +1143,10 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -1157,7 +1157,7 @@
         <v>34</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -1168,7 +1168,7 @@
         <v>38</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1179,7 +1179,7 @@
         <v>32</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1187,10 +1187,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -1200,7 +1200,7 @@
     </row>
     <row r="28" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -1224,7 +1224,7 @@
         <v>41</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1235,7 +1235,7 @@
         <v>44</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1243,10 +1243,10 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1257,7 +1257,7 @@
         <v>47</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1265,10 +1265,10 @@
         <v>0.6875</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>96</v>
+        <v>131</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1276,10 +1276,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -1289,7 +1289,7 @@
     </row>
     <row r="37" spans="1:3" ht="30" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -1310,10 +1310,10 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1321,10 +1321,10 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1332,10 +1332,10 @@
         <v>0.4375</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -1343,10 +1343,10 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -1354,7 +1354,7 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="C43" s="9"/>
     </row>
@@ -1363,10 +1363,10 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -1374,10 +1374,10 @@
         <v>0.6875</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -1385,10 +1385,10 @@
         <v>0.78472222222222221</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>